<commit_message>
Restrict caption files to individual masterfiles
</commit_message>
<xml_diff>
--- a/spec/fixtures/dropbox/example_batch_ingest/batch_manifest.xlsx
+++ b/spec/fixtures/dropbox/example_batch_ingest/batch_manifest.xlsx
@@ -73,6 +73,18 @@
     <t xml:space="preserve">Note Type</t>
   </si>
   <si>
+    <t xml:space="preserve">File</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Offset</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Date Digitized</t>
+  </si>
+  <si>
     <t xml:space="preserve">Caption File</t>
   </si>
   <si>
@@ -82,18 +94,6 @@
     <t xml:space="preserve">Caption Language</t>
   </si>
   <si>
-    <t xml:space="preserve">File</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Offset</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Label</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Date Digitized</t>
-  </si>
-  <si>
     <t xml:space="preserve">Skip Transcoding</t>
   </si>
   <si>
@@ -139,19 +139,19 @@
     <t xml:space="preserve">general</t>
   </si>
   <si>
+    <t xml:space="preserve">assets/sheephead_mountain.mov</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00:00:00.500</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quis quo</t>
+  </si>
+  <si>
     <t xml:space="preserve">assets/sheephead_mountain.mov.vtt</t>
   </si>
   <si>
     <t xml:space="preserve">Sheephead Captions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">assets/sheephead_mountain.mov</t>
-  </si>
-  <si>
-    <t xml:space="preserve">00:00:00.500</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quis quo</t>
   </si>
   <si>
     <t xml:space="preserve">Unde aliquid</t>
@@ -317,7 +317,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AG5"/>
-  <sheetFormatPr defaultColWidth="8.87109375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="20.37"/>
@@ -331,7 +331,7 @@
       <c r="B1" s="0" t="s">
         <v>1</v>
       </c>
-      <c r="T1" s="2"/>
+      <c r="Q1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
@@ -379,35 +379,35 @@
       <c r="O2" s="0" t="s">
         <v>16</v>
       </c>
-      <c r="P2" s="0" t="s">
+      <c r="P2" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="Q2" s="0" t="s">
+      <c r="Q2" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="R2" s="0" t="s">
+      <c r="R2" s="2" t="s">
         <v>19</v>
       </c>
       <c r="S2" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="T2" s="2" t="s">
+      <c r="T2" s="0" t="s">
         <v>21</v>
       </c>
-      <c r="U2" s="2" t="s">
+      <c r="U2" s="0" t="s">
         <v>22</v>
       </c>
-      <c r="V2" s="2" t="s">
+      <c r="V2" s="0" t="s">
         <v>23</v>
       </c>
       <c r="W2" s="2" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="X2" s="2" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="Y2" s="2" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="Z2" s="2" t="s">
         <v>24</v>
@@ -416,13 +416,13 @@
         <v>25</v>
       </c>
       <c r="AB2" s="2" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="AC2" s="0" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AD2" s="2" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="AE2" s="2" t="s">
         <v>24</v>
@@ -472,32 +472,32 @@
       <c r="O3" s="0" t="s">
         <v>38</v>
       </c>
-      <c r="P3" s="0" t="s">
+      <c r="P3" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="Q3" s="0" t="s">
+      <c r="Q3" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="R3" s="0" t="s">
+      <c r="R3" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="S3" s="3" t="n">
+        <v>42307</v>
+      </c>
+      <c r="T3" s="0" t="s">
+        <v>42</v>
+      </c>
+      <c r="U3" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="V3" s="0" t="s">
         <v>35</v>
       </c>
-      <c r="S3" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="T3" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="U3" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="V3" s="3" t="n">
-        <v>42307</v>
-      </c>
       <c r="W3" s="0" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="X3" s="2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="Y3" s="0" t="s">
         <v>44</v>
@@ -546,8 +546,8 @@
       <c r="O4" s="0" t="s">
         <v>56</v>
       </c>
-      <c r="S4" s="2" t="s">
-        <v>41</v>
+      <c r="P4" s="2" t="s">
+        <v>39</v>
       </c>
       <c r="Z4" s="0" t="s">
         <v>45</v>
@@ -566,8 +566,8 @@
       <c r="F5" s="0" t="s">
         <v>31</v>
       </c>
-      <c r="S5" s="2" t="s">
-        <v>41</v>
+      <c r="P5" s="2" t="s">
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add handling of transcript files to BatchIngest
</commit_message>
<xml_diff>
--- a/spec/fixtures/dropbox/example_batch_ingest/batch_manifest.xlsx
+++ b/spec/fixtures/dropbox/example_batch_ingest/batch_manifest.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="62">
   <si>
     <t xml:space="preserve">Frances Dickens</t>
   </si>
@@ -94,6 +94,15 @@
     <t xml:space="preserve">Caption Language</t>
   </si>
   <si>
+    <t xml:space="preserve">Transcript File</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transcript Label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Machine Generated</t>
+  </si>
+  <si>
     <t xml:space="preserve">Skip Transcoding</t>
   </si>
   <si>
@@ -154,10 +163,13 @@
     <t xml:space="preserve">Sheephead Captions</t>
   </si>
   <si>
+    <t xml:space="preserve">Sheephead Transcript</t>
+  </si>
+  <si>
+    <t xml:space="preserve">yes</t>
+  </si>
+  <si>
     <t xml:space="preserve">Unde aliquid</t>
-  </si>
-  <si>
-    <t xml:space="preserve">yes</t>
   </si>
   <si>
     <t xml:space="preserve">file:///tmp/sheephead_mountain_master.mov</t>
@@ -204,7 +216,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
@@ -234,6 +246,12 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -277,7 +295,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -291,6 +309,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -316,12 +338,12 @@
     <tabColor rgb="FFFFFFFF"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AG5"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:AJ5"/>
+  <sheetFormatPr defaultColWidth="8.8984375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="20.37"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="28" min="28" style="0" width="12.51"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="31" min="31" style="0" width="12.51"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -400,179 +422,197 @@
       <c r="V2" s="0" t="s">
         <v>23</v>
       </c>
-      <c r="W2" s="2" t="s">
+      <c r="W2" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="X2" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="Y2" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="Z2" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="X2" s="2" t="s">
+      <c r="AA2" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="Y2" s="2" t="s">
+      <c r="AB2" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="Z2" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="AA2" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="AB2" s="2" t="s">
+      <c r="AC2" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AD2" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="AE2" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="AC2" s="0" t="s">
+      <c r="AF2" s="0" t="s">
         <v>17</v>
       </c>
-      <c r="AD2" s="2" t="s">
+      <c r="AG2" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="AE2" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="AF2" s="0" t="s">
-        <v>26</v>
-      </c>
-      <c r="AG2" s="0" t="s">
+      <c r="AH2" s="2" t="s">
         <v>27</v>
+      </c>
+      <c r="AI2" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="AJ2" s="0" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C3" s="2" t="n">
         <v>2012</v>
       </c>
       <c r="D3" s="2"/>
       <c r="G3" s="0" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="I3" s="0" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="J3" s="0" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="K3" s="0" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="L3" s="0" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="M3" s="0" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="N3" s="0" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="O3" s="0" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="P3" s="2" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="Q3" s="2" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="R3" s="2" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="S3" s="3" t="n">
         <v>42307</v>
       </c>
       <c r="T3" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="U3" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="V3" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="W3" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="X3" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="Y3" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z3" s="0" t="s">
         <v>42</v>
       </c>
-      <c r="U3" s="0" t="s">
+      <c r="AA3" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="V3" s="0" t="s">
-        <v>35</v>
-      </c>
-      <c r="W3" s="0" t="s">
-        <v>39</v>
-      </c>
-      <c r="X3" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="Y3" s="0" t="s">
-        <v>44</v>
-      </c>
-      <c r="Z3" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="AA3" s="0" t="s">
-        <v>46</v>
-      </c>
-      <c r="AB3" s="4" t="n">
+      <c r="AB3" s="0" t="s">
+        <v>49</v>
+      </c>
+      <c r="AC3" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AD3" s="0" t="s">
+        <v>50</v>
+      </c>
+      <c r="AE3" s="5" t="n">
         <v>42308</v>
       </c>
-      <c r="AC3" s="0" t="s">
-        <v>47</v>
-      </c>
-      <c r="AD3" s="0" t="s">
-        <v>48</v>
-      </c>
-      <c r="AE3" s="0" t="s">
-        <v>49</v>
-      </c>
       <c r="AF3" s="0" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="AG3" s="0" t="s">
-        <v>51</v>
+        <v>52</v>
+      </c>
+      <c r="AH3" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI3" s="0" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ3" s="0" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="C4" s="0" t="n">
         <v>2011</v>
       </c>
       <c r="D4" s="0" t="s">
+        <v>58</v>
+      </c>
+      <c r="N4" s="0" t="s">
+        <v>59</v>
+      </c>
+      <c r="O4" s="0" t="s">
+        <v>60</v>
+      </c>
+      <c r="P4" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="AC4" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="AE4" s="5" t="n">
+        <v>42302</v>
+      </c>
+      <c r="AI4" s="0" t="s">
         <v>54</v>
-      </c>
-      <c r="N4" s="0" t="s">
-        <v>55</v>
-      </c>
-      <c r="O4" s="0" t="s">
-        <v>56</v>
-      </c>
-      <c r="P4" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="Z4" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="AB4" s="4" t="n">
-        <v>42302</v>
-      </c>
-      <c r="AF4" s="0" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E5" s="2" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="P5" s="2" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="AA3" r:id="rId1" display="file:///tmp/sheephead_mountain_master.mov"/>
+    <hyperlink ref="AD3" r:id="rId1" display="file:///tmp/sheephead_mountain_master.mov"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>